<commit_message>
v3 updates to cran
</commit_message>
<xml_diff>
--- a/data-raw/wcde-v3/indicator.xlsx
+++ b/data-raw/wcde-v3/indicator.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Guy\Dropbox\WCDE for Guy\meta\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\mig\Data Explorer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9EAD74E-5390-46E2-A667-96F8317B73C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF76A11B-6067-4EC7-A318-F45ACD3C9EF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="indicator" sheetId="1" r:id="rId1"/>
@@ -1344,27 +1344,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q36"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="50.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="50.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.1796875" customWidth="1"/>
-    <col min="6" max="6" width="5.26953125" customWidth="1"/>
+    <col min="5" max="5" width="4.140625" customWidth="1"/>
+    <col min="6" max="6" width="5.28515625" customWidth="1"/>
     <col min="7" max="7" width="5" customWidth="1"/>
     <col min="8" max="8" width="4" customWidth="1"/>
-    <col min="9" max="9" width="4.453125" customWidth="1"/>
-    <col min="10" max="10" width="7.7265625" customWidth="1"/>
-    <col min="11" max="11" width="6.81640625" customWidth="1"/>
-    <col min="12" max="12" width="4.7265625" customWidth="1"/>
-    <col min="13" max="13" width="7.26953125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.1796875" customWidth="1"/>
-    <col min="15" max="15" width="36.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.42578125" customWidth="1"/>
+    <col min="10" max="10" width="7.7109375" customWidth="1"/>
+    <col min="11" max="11" width="6.85546875" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.140625" customWidth="1"/>
+    <col min="15" max="15" width="36.5703125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="20" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="255.54296875" customWidth="1"/>
+    <col min="17" max="17" width="255.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>75</v>
       </c>
@@ -1417,7 +1417,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1452,7 +1452,7 @@
         <v>0</v>
       </c>
       <c r="L2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M2" s="1">
         <v>1</v>
@@ -1470,7 +1470,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>65</v>
       </c>
@@ -1505,7 +1505,7 @@
         <v>0</v>
       </c>
       <c r="L3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M3" s="1">
         <v>1</v>
@@ -1523,7 +1523,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>64</v>
       </c>
@@ -1558,7 +1558,7 @@
         <v>0</v>
       </c>
       <c r="L4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M4" s="1">
         <v>0</v>
@@ -1576,7 +1576,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -1611,7 +1611,7 @@
         <v>0</v>
       </c>
       <c r="L5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M5" s="1">
         <v>0</v>
@@ -1629,7 +1629,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>66</v>
       </c>
@@ -1664,7 +1664,7 @@
         <v>0</v>
       </c>
       <c r="L6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M6" s="1">
         <v>0</v>
@@ -1682,7 +1682,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>71</v>
       </c>
@@ -1717,7 +1717,7 @@
         <v>1</v>
       </c>
       <c r="L7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M7" s="1">
         <v>1</v>
@@ -1735,7 +1735,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>72</v>
       </c>
@@ -1770,7 +1770,7 @@
         <v>1</v>
       </c>
       <c r="L8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M8" s="1">
         <v>1</v>
@@ -1788,7 +1788,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -1823,7 +1823,7 @@
         <v>0</v>
       </c>
       <c r="L9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M9" s="1">
         <v>1</v>
@@ -1841,7 +1841,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -1876,7 +1876,7 @@
         <v>0</v>
       </c>
       <c r="L10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M10" s="1">
         <v>1</v>
@@ -1894,7 +1894,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -1929,7 +1929,7 @@
         <v>0</v>
       </c>
       <c r="L11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M11" s="1">
         <v>1</v>
@@ -1947,7 +1947,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -1982,7 +1982,7 @@
         <v>0</v>
       </c>
       <c r="L12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M12" s="1">
         <v>1</v>
@@ -2000,7 +2000,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -2035,7 +2035,7 @@
         <v>0</v>
       </c>
       <c r="L13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M13" s="1">
         <v>1</v>
@@ -2053,7 +2053,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>82</v>
       </c>
@@ -2088,7 +2088,7 @@
         <v>1</v>
       </c>
       <c r="L14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M14" s="1">
         <v>1</v>
@@ -2106,7 +2106,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>103</v>
       </c>
@@ -2141,7 +2141,7 @@
         <v>1</v>
       </c>
       <c r="L15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M15" s="1">
         <v>1</v>
@@ -2159,7 +2159,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -2194,7 +2194,7 @@
         <v>0</v>
       </c>
       <c r="L16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M16" s="1">
         <v>0</v>
@@ -2212,7 +2212,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -2247,7 +2247,7 @@
         <v>0</v>
       </c>
       <c r="L17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M17" s="1">
         <v>0</v>
@@ -2265,7 +2265,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>27</v>
       </c>
@@ -2300,7 +2300,7 @@
         <v>0</v>
       </c>
       <c r="L18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M18" s="1">
         <v>0</v>
@@ -2318,7 +2318,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>29</v>
       </c>
@@ -2353,7 +2353,7 @@
         <v>0</v>
       </c>
       <c r="L19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M19" s="1">
         <v>0</v>
@@ -2371,7 +2371,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>31</v>
       </c>
@@ -2406,7 +2406,7 @@
         <v>0</v>
       </c>
       <c r="L20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M20" s="1">
         <v>0</v>
@@ -2424,7 +2424,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>33</v>
       </c>
@@ -2459,7 +2459,7 @@
         <v>0</v>
       </c>
       <c r="L21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M21" s="1">
         <v>0</v>
@@ -2477,7 +2477,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>35</v>
       </c>
@@ -2512,7 +2512,7 @@
         <v>1</v>
       </c>
       <c r="L22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M22" s="1">
         <v>1</v>
@@ -2530,7 +2530,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>67</v>
       </c>
@@ -2583,7 +2583,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>37</v>
       </c>
@@ -2618,7 +2618,7 @@
         <v>1</v>
       </c>
       <c r="L24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M24" s="1">
         <v>1</v>
@@ -2636,7 +2636,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>39</v>
       </c>
@@ -2671,7 +2671,7 @@
         <v>1</v>
       </c>
       <c r="L25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M25" s="1">
         <v>1</v>
@@ -2689,7 +2689,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>41</v>
       </c>
@@ -2724,7 +2724,7 @@
         <v>1</v>
       </c>
       <c r="L26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M26" s="1">
         <v>1</v>
@@ -2742,7 +2742,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>43</v>
       </c>
@@ -2777,7 +2777,7 @@
         <v>1</v>
       </c>
       <c r="L27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M27" s="1">
         <v>1</v>
@@ -2795,7 +2795,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>45</v>
       </c>
@@ -2830,7 +2830,7 @@
         <v>1</v>
       </c>
       <c r="L28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M28" s="1">
         <v>1</v>
@@ -2848,7 +2848,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>47</v>
       </c>
@@ -2883,7 +2883,7 @@
         <v>1</v>
       </c>
       <c r="L29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M29" s="1">
         <v>1</v>
@@ -2901,7 +2901,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>86</v>
       </c>
@@ -2954,7 +2954,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>138</v>
       </c>
@@ -2989,7 +2989,7 @@
         <v>1</v>
       </c>
       <c r="L31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M31" s="1">
         <v>1</v>
@@ -3007,7 +3007,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>105</v>
       </c>
@@ -3060,7 +3060,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="33" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>134</v>
       </c>
@@ -3113,7 +3113,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="34" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>139</v>
       </c>
@@ -3166,7 +3166,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="35" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>140</v>
       </c>
@@ -3219,7 +3219,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="36" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>141</v>
       </c>

</xml_diff>